<commit_message>
[0300] Amended xlsx fields to use a nicer name
</commit_message>
<xml_diff>
--- a/lib/data/provider_seed_report_v_2.0_without_pii.xlsx
+++ b/lib/data/provider_seed_report_v_2.0_without_pii.xlsx
@@ -58,7 +58,7 @@
     <t xml:space="preserve">address__address_line_1</t>
   </si>
   <si>
-    <t xml:space="preserve">address_line_2</t>
+    <t xml:space="preserve">address__address_line_2</t>
   </si>
   <si>
     <t xml:space="preserve">address__address_line_3</t>
@@ -22994,43 +22994,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>